<commit_message>
improvements to reflectivity, xafs wheel, and change_edge
</commit_message>
<xml_diff>
--- a/startup/standards/standards.xlsx
+++ b/startup/standards/standards.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="12"/>
   </bookViews>
   <sheets>
     <sheet name="Ti" sheetId="1" state="visible" r:id="rId2"/>
@@ -1700,7 +1700,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3282" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3288" uniqueCount="600">
   <si>
     <t xml:space="preserve">Double wheel</t>
   </si>
@@ -3007,10 +3007,22 @@
     <t xml:space="preserve">PbCl, lead chloride</t>
   </si>
   <si>
+    <t xml:space="preserve">PtACAC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pt(C5H7O2)2, Platinum acetylacetonate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">powder on tape 18 layers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAS#15170=57=7. STREM Chemicals Inc., Cat#78-1400-1G, Lot#L00102507, Sample courtesy Elaine Flynn, Washington University</t>
+  </si>
+  <si>
     <t xml:space="preserve">PtRu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pt</t>
   </si>
   <si>
     <t xml:space="preserve">PtRu powder</t>
@@ -3850,7 +3862,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="111">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4199,6 +4211,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4374,9 +4390,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>40320</xdr:colOff>
+      <xdr:colOff>39960</xdr:colOff>
       <xdr:row>65</xdr:row>
-      <xdr:rowOff>66600</xdr:rowOff>
+      <xdr:rowOff>66240</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4389,8 +4405,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1656360" y="11943000"/>
-          <a:ext cx="3207240" cy="1822320"/>
+          <a:off x="1657080" y="11943000"/>
+          <a:ext cx="3206880" cy="1821960"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4416,9 +4432,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>855720</xdr:colOff>
+      <xdr:colOff>855360</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>162000</xdr:rowOff>
+      <xdr:rowOff>161640</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4431,8 +4447,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2073600" y="7088040"/>
-          <a:ext cx="3605400" cy="2246400"/>
+          <a:off x="2074320" y="7088040"/>
+          <a:ext cx="3605040" cy="2246040"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4458,9 +4474,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>855720</xdr:colOff>
+      <xdr:colOff>855360</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>162360</xdr:rowOff>
+      <xdr:rowOff>162000</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -4473,8 +4489,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2073600" y="5591880"/>
-          <a:ext cx="3605400" cy="2246760"/>
+          <a:off x="2074320" y="5591880"/>
+          <a:ext cx="3605040" cy="2246400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -4495,7 +4511,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -6709,7 +6725,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE30"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -8053,7 +8069,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE30"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -9379,7 +9395,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -11569,7 +11585,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -12555,7 +12571,7 @@
       <c r="AB24" s="62"/>
       <c r="AC24" s="63"/>
     </row>
-    <row r="25" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="43.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="69" t="n">
         <v>19</v>
       </c>
@@ -12565,16 +12581,28 @@
       <c r="D25" s="79" t="s">
         <v>3</v>
       </c>
-      <c r="E25" s="65"/>
+      <c r="E25" s="65" t="s">
+        <v>435</v>
+      </c>
       <c r="F25" s="66"/>
       <c r="G25" s="66"/>
       <c r="H25" s="66"/>
-      <c r="I25" s="67"/>
-      <c r="J25" s="68"/>
+      <c r="I25" s="67" t="s">
+        <v>436</v>
+      </c>
+      <c r="J25" s="68" t="s">
+        <v>164</v>
+      </c>
       <c r="K25" s="69"/>
-      <c r="L25" s="86"/>
-      <c r="M25" s="71"/>
-      <c r="N25" s="73"/>
+      <c r="L25" s="87" t="s">
+        <v>437</v>
+      </c>
+      <c r="M25" s="53" t="s">
+        <v>438</v>
+      </c>
+      <c r="N25" s="73" t="s">
+        <v>439</v>
+      </c>
       <c r="O25" s="64"/>
       <c r="P25" s="29"/>
       <c r="Q25" s="57"/>
@@ -12624,7 +12652,7 @@
         <v>3</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>435</v>
+        <v>440</v>
       </c>
       <c r="I27" s="67" t="s">
         <v>436</v>
@@ -12633,7 +12661,7 @@
         <v>164</v>
       </c>
       <c r="L27" s="0" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="M27" s="71" t="s">
         <v>53</v>
@@ -12666,7 +12694,7 @@
         <v>3</v>
       </c>
       <c r="E28" s="65" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="F28" s="66"/>
       <c r="G28" s="66"/>
@@ -12679,13 +12707,13 @@
       </c>
       <c r="K28" s="69"/>
       <c r="L28" s="86" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="M28" s="71" t="s">
         <v>53</v>
       </c>
       <c r="N28" s="72" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="O28" s="64"/>
       <c r="P28" s="29"/>
@@ -12712,7 +12740,7 @@
         <v>3</v>
       </c>
       <c r="E29" s="65" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="F29" s="66"/>
       <c r="G29" s="66"/>
@@ -12725,13 +12753,13 @@
       </c>
       <c r="K29" s="69"/>
       <c r="L29" s="70" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="M29" s="71" t="s">
         <v>53</v>
       </c>
       <c r="N29" s="72" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="O29" s="64"/>
       <c r="P29" s="29"/>
@@ -12758,7 +12786,7 @@
         <v>3</v>
       </c>
       <c r="E30" s="65" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="F30" s="66"/>
       <c r="G30" s="66"/>
@@ -12771,13 +12799,13 @@
       </c>
       <c r="K30" s="69"/>
       <c r="L30" s="65" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="M30" s="71" t="s">
         <v>53</v>
       </c>
       <c r="N30" s="72" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="O30" s="64"/>
       <c r="P30" s="29"/>
@@ -12838,20 +12866,20 @@
         <v>3</v>
       </c>
       <c r="E32" s="71" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="F32" s="66"/>
       <c r="G32" s="66"/>
       <c r="H32" s="66"/>
       <c r="I32" s="67" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="J32" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K32" s="69"/>
       <c r="L32" s="70" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="M32" s="71"/>
       <c r="N32" s="73" t="s">
@@ -12882,20 +12910,20 @@
         <v>3</v>
       </c>
       <c r="E33" s="65" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="F33" s="66"/>
       <c r="G33" s="66"/>
       <c r="H33" s="66"/>
       <c r="I33" s="67" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="J33" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K33" s="69"/>
       <c r="L33" s="70" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="M33" s="71" t="s">
         <v>53</v>
@@ -13132,20 +13160,20 @@
         <v>3</v>
       </c>
       <c r="E40" s="65" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="F40" s="66"/>
       <c r="G40" s="66"/>
       <c r="H40" s="66"/>
       <c r="I40" s="67" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="J40" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K40" s="69"/>
       <c r="L40" s="70" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="M40" s="71" t="s">
         <v>53</v>
@@ -13176,20 +13204,20 @@
         <v>3</v>
       </c>
       <c r="E41" s="65" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="F41" s="66"/>
       <c r="G41" s="66"/>
       <c r="H41" s="66"/>
       <c r="I41" s="67" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="J41" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K41" s="69"/>
       <c r="L41" s="70" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="M41" s="71" t="s">
         <v>53</v>
@@ -13220,20 +13248,20 @@
         <v>3</v>
       </c>
       <c r="E42" s="65" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="F42" s="66"/>
       <c r="G42" s="66"/>
       <c r="H42" s="66"/>
       <c r="I42" s="67" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="J42" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K42" s="69"/>
       <c r="L42" s="70" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
       <c r="M42" s="71" t="s">
         <v>53</v>
@@ -13264,20 +13292,20 @@
         <v>3</v>
       </c>
       <c r="E43" s="65" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="F43" s="66"/>
       <c r="G43" s="66"/>
       <c r="H43" s="66"/>
       <c r="I43" s="67" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="J43" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K43" s="69"/>
       <c r="L43" s="70" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="M43" s="71" t="s">
         <v>53</v>
@@ -13383,20 +13411,20 @@
         <v>3</v>
       </c>
       <c r="E47" s="65" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="F47" s="66"/>
       <c r="G47" s="66"/>
       <c r="H47" s="66"/>
       <c r="I47" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J47" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K47" s="69"/>
       <c r="L47" s="70" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="M47" s="71" t="s">
         <v>53</v>
@@ -13427,20 +13455,20 @@
         <v>3</v>
       </c>
       <c r="E48" s="65" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="F48" s="66"/>
       <c r="G48" s="66"/>
       <c r="H48" s="66"/>
       <c r="I48" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J48" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K48" s="69"/>
       <c r="L48" s="86" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="M48" s="71" t="s">
         <v>393</v>
@@ -13505,20 +13533,20 @@
         <v>3</v>
       </c>
       <c r="E50" s="65" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="F50" s="66"/>
       <c r="G50" s="66"/>
       <c r="H50" s="66"/>
       <c r="I50" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J50" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K50" s="69"/>
       <c r="L50" s="70" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="M50" s="71" t="s">
         <v>393</v>
@@ -13549,20 +13577,20 @@
         <v>3</v>
       </c>
       <c r="E51" s="65" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="F51" s="66"/>
       <c r="G51" s="66"/>
       <c r="H51" s="66"/>
       <c r="I51" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J51" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K51" s="69"/>
       <c r="L51" s="70" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="M51" s="71" t="s">
         <v>393</v>
@@ -13593,24 +13621,24 @@
         <v>3</v>
       </c>
       <c r="E52" s="65" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="F52" s="66"/>
       <c r="G52" s="66"/>
       <c r="H52" s="66"/>
       <c r="I52" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J52" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K52" s="69"/>
       <c r="L52" s="65" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="M52" s="71"/>
       <c r="N52" s="73" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="O52" s="64"/>
       <c r="P52" s="29"/>
@@ -13637,20 +13665,20 @@
         <v>3</v>
       </c>
       <c r="E53" s="65" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="F53" s="66"/>
       <c r="G53" s="66"/>
       <c r="H53" s="66"/>
       <c r="I53" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J53" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K53" s="69"/>
       <c r="L53" s="70" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="M53" s="65"/>
       <c r="N53" s="73" t="s">
@@ -13681,20 +13709,20 @@
         <v>3</v>
       </c>
       <c r="E54" s="65" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="F54" s="66"/>
       <c r="G54" s="66"/>
       <c r="H54" s="66"/>
       <c r="I54" s="67" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="J54" s="68" t="s">
         <v>164</v>
       </c>
       <c r="K54" s="69"/>
       <c r="L54" s="70" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="M54" s="71"/>
       <c r="N54" s="73" t="s">
@@ -13831,7 +13859,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE79"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -14180,26 +14208,26 @@
         <v>3</v>
       </c>
       <c r="E7" s="53" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="F7" s="13"/>
       <c r="G7" s="13"/>
       <c r="H7" s="13"/>
-      <c r="I7" s="87" t="s">
+      <c r="I7" s="88" t="s">
         <v>49</v>
       </c>
-      <c r="J7" s="88" t="s">
+      <c r="J7" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K7" s="50"/>
       <c r="L7" s="56" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="M7" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N7" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O7" s="56"/>
       <c r="P7" s="29"/>
@@ -14226,20 +14254,20 @@
         <v>3</v>
       </c>
       <c r="E8" s="53" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-      <c r="I8" s="87" t="s">
-        <v>477</v>
-      </c>
-      <c r="J8" s="88" t="s">
+      <c r="I8" s="88" t="s">
+        <v>481</v>
+      </c>
+      <c r="J8" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K8" s="50"/>
       <c r="L8" s="56" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="M8" s="53" t="s">
         <v>108</v>
@@ -14248,7 +14276,7 @@
         <v>167</v>
       </c>
       <c r="O8" s="75" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="P8" s="29"/>
       <c r="Q8" s="57"/>
@@ -14264,36 +14292,36 @@
       <c r="AC8" s="63"/>
     </row>
     <row r="9" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="89" t="n">
+      <c r="B9" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="91" t="s">
+      <c r="C9" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E9" s="92" t="s">
-        <v>480</v>
-      </c>
-      <c r="F9" s="89"/>
-      <c r="G9" s="89"/>
-      <c r="H9" s="89"/>
-      <c r="I9" s="93" t="s">
-        <v>481</v>
-      </c>
-      <c r="J9" s="94" t="s">
+      <c r="E9" s="93" t="s">
+        <v>484</v>
+      </c>
+      <c r="F9" s="90"/>
+      <c r="G9" s="90"/>
+      <c r="H9" s="90"/>
+      <c r="I9" s="94" t="s">
+        <v>485</v>
+      </c>
+      <c r="J9" s="95" t="s">
         <v>164</v>
       </c>
-      <c r="K9" s="89"/>
-      <c r="L9" s="95" t="s">
-        <v>482</v>
-      </c>
-      <c r="M9" s="92"/>
-      <c r="N9" s="96"/>
-      <c r="O9" s="95"/>
-      <c r="P9" s="97"/>
-      <c r="Q9" s="95"/>
+      <c r="K9" s="90"/>
+      <c r="L9" s="96" t="s">
+        <v>486</v>
+      </c>
+      <c r="M9" s="93"/>
+      <c r="N9" s="97"/>
+      <c r="O9" s="96"/>
+      <c r="P9" s="98"/>
+      <c r="Q9" s="96"/>
       <c r="R9" s="58"/>
       <c r="U9" s="12"/>
       <c r="V9" s="59"/>
@@ -14316,15 +14344,15 @@
         <v>3</v>
       </c>
       <c r="E10" s="53" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="F10" s="13"/>
       <c r="G10" s="13"/>
       <c r="H10" s="13"/>
-      <c r="I10" s="87" t="s">
+      <c r="I10" s="88" t="s">
         <v>243</v>
       </c>
-      <c r="J10" s="88" t="s">
+      <c r="J10" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K10" s="50"/>
@@ -14335,7 +14363,7 @@
         <v>329</v>
       </c>
       <c r="N10" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O10" s="56"/>
       <c r="P10" s="29"/>
@@ -14362,20 +14390,20 @@
         <v>3</v>
       </c>
       <c r="E11" s="53" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="F11" s="13"/>
       <c r="G11" s="13"/>
       <c r="H11" s="13"/>
-      <c r="I11" s="87" t="s">
+      <c r="I11" s="88" t="s">
         <v>176</v>
       </c>
-      <c r="J11" s="88" t="s">
+      <c r="J11" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K11" s="50"/>
       <c r="L11" s="56" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="M11" s="53" t="s">
         <v>108</v>
@@ -14384,7 +14412,7 @@
         <v>167</v>
       </c>
       <c r="O11" s="75" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="P11" s="29"/>
       <c r="Q11" s="57"/>
@@ -14410,20 +14438,20 @@
         <v>3</v>
       </c>
       <c r="E12" s="53" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="F12" s="13"/>
       <c r="G12" s="13"/>
       <c r="H12" s="13"/>
-      <c r="I12" s="87" t="s">
-        <v>477</v>
-      </c>
-      <c r="J12" s="88" t="s">
-        <v>487</v>
+      <c r="I12" s="88" t="s">
+        <v>481</v>
+      </c>
+      <c r="J12" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K12" s="50"/>
       <c r="L12" s="56" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="M12" s="53" t="s">
         <v>108</v>
@@ -14456,15 +14484,15 @@
         <v>3</v>
       </c>
       <c r="E13" s="53" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="F13" s="13"/>
       <c r="G13" s="13"/>
       <c r="H13" s="13"/>
-      <c r="I13" s="87" t="s">
+      <c r="I13" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="J13" s="88" t="s">
+      <c r="J13" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K13" s="50"/>
@@ -14478,7 +14506,7 @@
         <v>167</v>
       </c>
       <c r="O13" s="75" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="P13" s="29"/>
       <c r="Q13" s="57"/>
@@ -14504,20 +14532,20 @@
         <v>3</v>
       </c>
       <c r="E14" s="53" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="F14" s="13"/>
       <c r="G14" s="13"/>
       <c r="H14" s="13"/>
-      <c r="I14" s="87" t="s">
+      <c r="I14" s="88" t="s">
         <v>200</v>
       </c>
-      <c r="J14" s="88" t="s">
+      <c r="J14" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K14" s="50"/>
       <c r="L14" s="56" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="M14" s="53" t="s">
         <v>108</v>
@@ -14552,26 +14580,26 @@
         <v>3</v>
       </c>
       <c r="E15" s="53" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="F15" s="13"/>
       <c r="G15" s="13"/>
       <c r="H15" s="13"/>
-      <c r="I15" s="87" t="s">
-        <v>493</v>
-      </c>
-      <c r="J15" s="88" t="s">
+      <c r="I15" s="88" t="s">
+        <v>497</v>
+      </c>
+      <c r="J15" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K15" s="50"/>
       <c r="L15" s="56" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="M15" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N15" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O15" s="56"/>
       <c r="P15" s="29"/>
@@ -14588,36 +14616,36 @@
       <c r="AC15" s="63"/>
     </row>
     <row r="16" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="89" t="n">
+      <c r="B16" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="91" t="s">
+      <c r="C16" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E16" s="92" t="s">
-        <v>480</v>
-      </c>
-      <c r="F16" s="89"/>
-      <c r="G16" s="89"/>
-      <c r="H16" s="89"/>
-      <c r="I16" s="93" t="s">
-        <v>481</v>
-      </c>
-      <c r="J16" s="94" t="s">
-        <v>487</v>
-      </c>
-      <c r="K16" s="89"/>
-      <c r="L16" s="95" t="s">
-        <v>482</v>
-      </c>
-      <c r="M16" s="92"/>
-      <c r="N16" s="96"/>
-      <c r="O16" s="95"/>
-      <c r="P16" s="97"/>
-      <c r="Q16" s="95"/>
+      <c r="E16" s="93" t="s">
+        <v>484</v>
+      </c>
+      <c r="F16" s="90"/>
+      <c r="G16" s="90"/>
+      <c r="H16" s="90"/>
+      <c r="I16" s="94" t="s">
+        <v>485</v>
+      </c>
+      <c r="J16" s="95" t="s">
+        <v>491</v>
+      </c>
+      <c r="K16" s="90"/>
+      <c r="L16" s="96" t="s">
+        <v>486</v>
+      </c>
+      <c r="M16" s="93"/>
+      <c r="N16" s="97"/>
+      <c r="O16" s="96"/>
+      <c r="P16" s="98"/>
+      <c r="Q16" s="96"/>
       <c r="R16" s="58"/>
       <c r="U16" s="12"/>
       <c r="V16" s="59"/>
@@ -14640,20 +14668,20 @@
         <v>3</v>
       </c>
       <c r="E17" s="53" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="13"/>
       <c r="H17" s="13"/>
-      <c r="I17" s="87" t="s">
+      <c r="I17" s="88" t="s">
         <v>205</v>
       </c>
-      <c r="J17" s="88" t="s">
+      <c r="J17" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K17" s="50"/>
       <c r="L17" s="56" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="M17" s="53" t="s">
         <v>108</v>
@@ -14688,20 +14716,20 @@
         <v>3</v>
       </c>
       <c r="E18" s="53" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="F18" s="13"/>
       <c r="G18" s="13"/>
       <c r="H18" s="13"/>
-      <c r="I18" s="87" t="s">
+      <c r="I18" s="88" t="s">
         <v>176</v>
       </c>
-      <c r="J18" s="88" t="s">
-        <v>487</v>
+      <c r="J18" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K18" s="50"/>
       <c r="L18" s="56" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="M18" s="53" t="s">
         <v>108</v>
@@ -14734,26 +14762,26 @@
         <v>3</v>
       </c>
       <c r="E19" s="53" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="F19" s="13"/>
       <c r="G19" s="13"/>
       <c r="H19" s="13"/>
-      <c r="I19" s="87" t="s">
+      <c r="I19" s="88" t="s">
         <v>271</v>
       </c>
-      <c r="J19" s="88" t="s">
+      <c r="J19" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K19" s="50"/>
       <c r="L19" s="56" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="M19" s="53" t="s">
         <v>255</v>
       </c>
       <c r="N19" s="86" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="O19" s="56"/>
       <c r="P19" s="29"/>
@@ -14780,16 +14808,16 @@
         <v>3</v>
       </c>
       <c r="E20" s="53" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="F20" s="13"/>
       <c r="G20" s="13"/>
       <c r="H20" s="13"/>
-      <c r="I20" s="87" t="s">
+      <c r="I20" s="88" t="s">
         <v>163</v>
       </c>
-      <c r="J20" s="88" t="s">
-        <v>487</v>
+      <c r="J20" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K20" s="50"/>
       <c r="L20" s="56" t="s">
@@ -14826,20 +14854,20 @@
         <v>3</v>
       </c>
       <c r="E21" s="53" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="F21" s="13"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13"/>
-      <c r="I21" s="87" t="s">
+      <c r="I21" s="88" t="s">
         <v>179</v>
       </c>
-      <c r="J21" s="88" t="s">
+      <c r="J21" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K21" s="50"/>
       <c r="L21" s="56" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="M21" s="53" t="s">
         <v>108</v>
@@ -14874,20 +14902,20 @@
         <v>3</v>
       </c>
       <c r="E22" s="53" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="F22" s="13"/>
       <c r="G22" s="13"/>
       <c r="H22" s="13"/>
-      <c r="I22" s="87" t="s">
+      <c r="I22" s="88" t="s">
         <v>200</v>
       </c>
-      <c r="J22" s="88" t="s">
-        <v>487</v>
+      <c r="J22" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K22" s="50"/>
       <c r="L22" s="56" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="M22" s="53" t="s">
         <v>108</v>
@@ -14920,20 +14948,20 @@
         <v>3</v>
       </c>
       <c r="E23" s="53" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="F23" s="13"/>
       <c r="G23" s="13"/>
       <c r="H23" s="13"/>
-      <c r="I23" s="87" t="s">
+      <c r="I23" s="88" t="s">
         <v>183</v>
       </c>
-      <c r="J23" s="88" t="s">
+      <c r="J23" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K23" s="50"/>
       <c r="L23" s="56" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="M23" s="53" t="s">
         <v>108</v>
@@ -14968,26 +14996,26 @@
         <v>3</v>
       </c>
       <c r="E24" s="53" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="F24" s="13"/>
       <c r="G24" s="13"/>
       <c r="H24" s="13"/>
-      <c r="I24" s="87" t="s">
+      <c r="I24" s="88" t="s">
         <v>89</v>
       </c>
-      <c r="J24" s="88" t="s">
+      <c r="J24" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K24" s="50"/>
       <c r="L24" s="56" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="M24" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N24" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O24" s="56"/>
       <c r="P24" s="29"/>
@@ -15014,20 +15042,20 @@
         <v>3</v>
       </c>
       <c r="E25" s="53" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="F25" s="13"/>
       <c r="G25" s="13"/>
       <c r="H25" s="13"/>
-      <c r="I25" s="87" t="s">
+      <c r="I25" s="88" t="s">
         <v>205</v>
       </c>
-      <c r="J25" s="88" t="s">
-        <v>487</v>
+      <c r="J25" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K25" s="50"/>
       <c r="L25" s="56" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="M25" s="53" t="s">
         <v>108</v>
@@ -15060,20 +15088,20 @@
         <v>3</v>
       </c>
       <c r="E26" s="53" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="F26" s="13"/>
       <c r="G26" s="13"/>
       <c r="H26" s="13"/>
-      <c r="I26" s="87" t="s">
+      <c r="I26" s="88" t="s">
         <v>195</v>
       </c>
-      <c r="J26" s="88" t="s">
+      <c r="J26" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K26" s="50"/>
       <c r="L26" s="56" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="M26" s="53" t="s">
         <v>108</v>
@@ -15108,20 +15136,20 @@
         <v>3</v>
       </c>
       <c r="E27" s="53" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="F27" s="13"/>
       <c r="G27" s="13"/>
       <c r="H27" s="13"/>
-      <c r="I27" s="87" t="s">
+      <c r="I27" s="88" t="s">
         <v>219</v>
       </c>
-      <c r="J27" s="88" t="s">
+      <c r="J27" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K27" s="50"/>
       <c r="L27" s="56" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="M27" s="53" t="s">
         <v>108</v>
@@ -15156,26 +15184,26 @@
         <v>3</v>
       </c>
       <c r="E28" s="53" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="13"/>
       <c r="H28" s="13"/>
-      <c r="I28" s="87" t="s">
+      <c r="I28" s="88" t="s">
         <v>305</v>
       </c>
-      <c r="J28" s="88" t="s">
+      <c r="J28" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K28" s="50"/>
       <c r="L28" s="56" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="M28" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N28" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O28" s="56"/>
       <c r="P28" s="29"/>
@@ -15202,20 +15230,20 @@
         <v>3</v>
       </c>
       <c r="E29" s="53" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="13"/>
       <c r="H29" s="13"/>
-      <c r="I29" s="87" t="s">
+      <c r="I29" s="88" t="s">
         <v>179</v>
       </c>
-      <c r="J29" s="88" t="s">
-        <v>487</v>
+      <c r="J29" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K29" s="50"/>
       <c r="L29" s="56" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="M29" s="53" t="s">
         <v>108</v>
@@ -15248,20 +15276,20 @@
         <v>3</v>
       </c>
       <c r="E30" s="53" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="13"/>
       <c r="H30" s="13"/>
-      <c r="I30" s="87" t="s">
+      <c r="I30" s="88" t="s">
         <v>222</v>
       </c>
-      <c r="J30" s="88" t="s">
+      <c r="J30" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K30" s="50"/>
       <c r="L30" s="56" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="M30" s="53" t="s">
         <v>108</v>
@@ -15296,20 +15324,20 @@
         <v>3</v>
       </c>
       <c r="E31" s="53" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="13"/>
       <c r="H31" s="13"/>
-      <c r="I31" s="87" t="s">
+      <c r="I31" s="88" t="s">
         <v>183</v>
       </c>
-      <c r="J31" s="88" t="s">
-        <v>487</v>
+      <c r="J31" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K31" s="50"/>
       <c r="L31" s="56" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="M31" s="53" t="s">
         <v>108</v>
@@ -15342,20 +15370,20 @@
         <v>3</v>
       </c>
       <c r="E32" s="53" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="F32" s="13"/>
       <c r="G32" s="13"/>
       <c r="H32" s="13"/>
-      <c r="I32" s="87" t="s">
+      <c r="I32" s="88" t="s">
         <v>225</v>
       </c>
-      <c r="J32" s="88" t="s">
+      <c r="J32" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K32" s="50"/>
       <c r="L32" s="56" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="M32" s="53" t="s">
         <v>108</v>
@@ -15390,26 +15418,26 @@
         <v>3</v>
       </c>
       <c r="E33" s="53" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="13"/>
       <c r="H33" s="13"/>
-      <c r="I33" s="87" t="s">
+      <c r="I33" s="88" t="s">
         <v>313</v>
       </c>
-      <c r="J33" s="88" t="s">
+      <c r="J33" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K33" s="50"/>
       <c r="L33" s="56" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="M33" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N33" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O33" s="56"/>
       <c r="P33" s="29"/>
@@ -15436,15 +15464,15 @@
         <v>3</v>
       </c>
       <c r="E34" s="53" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="F34" s="13"/>
       <c r="G34" s="13"/>
       <c r="H34" s="13"/>
-      <c r="I34" s="87" t="s">
+      <c r="I34" s="88" t="s">
         <v>190</v>
       </c>
-      <c r="J34" s="88" t="s">
+      <c r="J34" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K34" s="50"/>
@@ -15482,20 +15510,20 @@
         <v>3</v>
       </c>
       <c r="E35" s="53" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="F35" s="13"/>
       <c r="G35" s="13"/>
       <c r="H35" s="13"/>
-      <c r="I35" s="87" t="s">
+      <c r="I35" s="88" t="s">
         <v>195</v>
       </c>
-      <c r="J35" s="88" t="s">
-        <v>487</v>
+      <c r="J35" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K35" s="50"/>
       <c r="L35" s="56" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="M35" s="53" t="s">
         <v>108</v>
@@ -15528,20 +15556,20 @@
         <v>3</v>
       </c>
       <c r="E36" s="53" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="F36" s="13"/>
       <c r="G36" s="13"/>
       <c r="H36" s="13"/>
-      <c r="I36" s="87" t="s">
+      <c r="I36" s="88" t="s">
         <v>228</v>
       </c>
-      <c r="J36" s="88" t="s">
+      <c r="J36" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K36" s="50"/>
       <c r="L36" s="56" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="M36" s="53" t="s">
         <v>108</v>
@@ -15574,20 +15602,20 @@
         <v>3</v>
       </c>
       <c r="E37" s="53" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="F37" s="13"/>
       <c r="G37" s="13"/>
       <c r="H37" s="13"/>
-      <c r="I37" s="87" t="s">
+      <c r="I37" s="88" t="s">
         <v>219</v>
       </c>
-      <c r="J37" s="88" t="s">
-        <v>487</v>
+      <c r="J37" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K37" s="50"/>
       <c r="L37" s="56" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="M37" s="53" t="s">
         <v>108</v>
@@ -15620,15 +15648,15 @@
         <v>3</v>
       </c>
       <c r="E38" s="53" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="F38" s="13"/>
       <c r="G38" s="13"/>
       <c r="H38" s="13"/>
-      <c r="I38" s="87" t="s">
+      <c r="I38" s="88" t="s">
         <v>192</v>
       </c>
-      <c r="J38" s="88" t="s">
+      <c r="J38" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K38" s="50"/>
@@ -15666,26 +15694,26 @@
         <v>3</v>
       </c>
       <c r="E39" s="53" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="F39" s="13"/>
       <c r="G39" s="13"/>
       <c r="H39" s="13"/>
-      <c r="I39" s="87" t="s">
+      <c r="I39" s="88" t="s">
         <v>326</v>
       </c>
-      <c r="J39" s="88" t="s">
+      <c r="J39" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K39" s="50"/>
       <c r="L39" s="56" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="M39" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N39" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O39" s="56"/>
       <c r="P39" s="29"/>
@@ -15712,20 +15740,20 @@
         <v>3</v>
       </c>
       <c r="E40" s="53" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="F40" s="13"/>
       <c r="G40" s="13"/>
       <c r="H40" s="13"/>
-      <c r="I40" s="87" t="s">
+      <c r="I40" s="88" t="s">
         <v>222</v>
       </c>
-      <c r="J40" s="88" t="s">
-        <v>487</v>
+      <c r="J40" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K40" s="50"/>
       <c r="L40" s="56" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="M40" s="53" t="s">
         <v>108</v>
@@ -15758,20 +15786,20 @@
         <v>3</v>
       </c>
       <c r="E41" s="53" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="F41" s="13"/>
       <c r="G41" s="13"/>
       <c r="H41" s="13"/>
-      <c r="I41" s="87" t="s">
+      <c r="I41" s="88" t="s">
         <v>232</v>
       </c>
-      <c r="J41" s="88" t="s">
+      <c r="J41" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K41" s="50"/>
       <c r="L41" s="56" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="M41" s="53" t="s">
         <v>108</v>
@@ -15804,20 +15832,20 @@
         <v>3</v>
       </c>
       <c r="E42" s="53" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="F42" s="13"/>
       <c r="G42" s="13"/>
       <c r="H42" s="13"/>
-      <c r="I42" s="87" t="s">
+      <c r="I42" s="88" t="s">
         <v>225</v>
       </c>
-      <c r="J42" s="88" t="s">
-        <v>487</v>
+      <c r="J42" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K42" s="50"/>
       <c r="L42" s="56" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="M42" s="53" t="s">
         <v>108</v>
@@ -15850,20 +15878,20 @@
         <v>3</v>
       </c>
       <c r="E43" s="53" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="F43" s="13"/>
       <c r="G43" s="13"/>
       <c r="H43" s="13"/>
-      <c r="I43" s="87" t="s">
-        <v>527</v>
-      </c>
-      <c r="J43" s="88" t="s">
+      <c r="I43" s="88" t="s">
+        <v>531</v>
+      </c>
+      <c r="J43" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K43" s="50"/>
       <c r="L43" s="56" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="M43" s="53" t="s">
         <v>108</v>
@@ -15896,26 +15924,26 @@
         <v>3</v>
       </c>
       <c r="E44" s="53" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="F44" s="13"/>
       <c r="G44" s="13"/>
       <c r="H44" s="13"/>
-      <c r="I44" s="87" t="s">
+      <c r="I44" s="88" t="s">
         <v>324</v>
       </c>
-      <c r="J44" s="88" t="s">
+      <c r="J44" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K44" s="50"/>
       <c r="L44" s="56" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="M44" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N44" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="O44" s="56"/>
       <c r="P44" s="29"/>
@@ -15942,16 +15970,16 @@
         <v>3</v>
       </c>
       <c r="E45" s="53" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="F45" s="13"/>
       <c r="G45" s="13"/>
       <c r="H45" s="13"/>
-      <c r="I45" s="87" t="s">
+      <c r="I45" s="88" t="s">
         <v>190</v>
       </c>
-      <c r="J45" s="88" t="s">
-        <v>487</v>
+      <c r="J45" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K45" s="50"/>
       <c r="L45" s="56" t="s">
@@ -15988,20 +16016,20 @@
         <v>3</v>
       </c>
       <c r="E46" s="53" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="F46" s="13"/>
       <c r="G46" s="13"/>
       <c r="H46" s="13"/>
-      <c r="I46" s="87" t="s">
-        <v>532</v>
-      </c>
-      <c r="J46" s="88" t="s">
+      <c r="I46" s="88" t="s">
+        <v>536</v>
+      </c>
+      <c r="J46" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K46" s="50"/>
       <c r="L46" s="56" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="M46" s="53" t="s">
         <v>108</v>
@@ -16034,20 +16062,20 @@
         <v>3</v>
       </c>
       <c r="E47" s="53" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="F47" s="13"/>
       <c r="G47" s="13"/>
       <c r="H47" s="13"/>
-      <c r="I47" s="87" t="s">
+      <c r="I47" s="88" t="s">
         <v>228</v>
       </c>
-      <c r="J47" s="88" t="s">
-        <v>487</v>
+      <c r="J47" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K47" s="50"/>
       <c r="L47" s="56" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="M47" s="53" t="s">
         <v>108</v>
@@ -16080,20 +16108,20 @@
         <v>3</v>
       </c>
       <c r="E48" s="53" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="F48" s="13"/>
       <c r="G48" s="13"/>
       <c r="H48" s="13"/>
-      <c r="I48" s="87" t="s">
-        <v>535</v>
-      </c>
-      <c r="J48" s="88" t="s">
+      <c r="I48" s="88" t="s">
+        <v>539</v>
+      </c>
+      <c r="J48" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K48" s="50"/>
       <c r="L48" s="56" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="M48" s="53" t="s">
         <v>108</v>
@@ -16126,20 +16154,20 @@
         <v>3</v>
       </c>
       <c r="E49" s="53" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="F49" s="13"/>
       <c r="G49" s="13"/>
       <c r="H49" s="13"/>
-      <c r="I49" s="87" t="s">
-        <v>538</v>
-      </c>
-      <c r="J49" s="88" t="s">
+      <c r="I49" s="88" t="s">
+        <v>542</v>
+      </c>
+      <c r="J49" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K49" s="50"/>
       <c r="L49" s="56" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="M49" s="53" t="s">
         <v>108</v>
@@ -16172,16 +16200,16 @@
         <v>3</v>
       </c>
       <c r="E50" s="53" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="F50" s="13"/>
       <c r="G50" s="13"/>
       <c r="H50" s="13"/>
-      <c r="I50" s="87" t="s">
+      <c r="I50" s="88" t="s">
         <v>192</v>
       </c>
-      <c r="J50" s="88" t="s">
-        <v>487</v>
+      <c r="J50" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K50" s="50"/>
       <c r="L50" s="56" t="s">
@@ -16218,20 +16246,20 @@
         <v>3</v>
       </c>
       <c r="E51" s="53" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="F51" s="13"/>
       <c r="G51" s="13"/>
       <c r="H51" s="13"/>
-      <c r="I51" s="87" t="s">
-        <v>450</v>
-      </c>
-      <c r="J51" s="88" t="s">
+      <c r="I51" s="88" t="s">
+        <v>454</v>
+      </c>
+      <c r="J51" s="89" t="s">
         <v>164</v>
       </c>
       <c r="K51" s="50"/>
       <c r="L51" s="56" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="M51" s="86" t="s">
         <v>53</v>
@@ -16262,20 +16290,20 @@
         <v>3</v>
       </c>
       <c r="E52" s="53" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="F52" s="13"/>
       <c r="G52" s="13"/>
       <c r="H52" s="13"/>
-      <c r="I52" s="87" t="s">
+      <c r="I52" s="88" t="s">
         <v>232</v>
       </c>
-      <c r="J52" s="88" t="s">
-        <v>487</v>
+      <c r="J52" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="K52" s="50"/>
       <c r="L52" s="56" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="M52" s="53" t="s">
         <v>108</v>
@@ -16298,36 +16326,36 @@
       <c r="AC52" s="63"/>
     </row>
     <row r="53" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="89" t="n">
+      <c r="B53" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C53" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D53" s="91" t="s">
+      <c r="C53" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D53" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E53" s="92" t="s">
-        <v>541</v>
-      </c>
-      <c r="F53" s="89"/>
-      <c r="G53" s="89"/>
-      <c r="H53" s="89"/>
-      <c r="I53" s="93" t="s">
-        <v>542</v>
-      </c>
-      <c r="J53" s="94" t="s">
+      <c r="E53" s="93" t="s">
+        <v>545</v>
+      </c>
+      <c r="F53" s="90"/>
+      <c r="G53" s="90"/>
+      <c r="H53" s="90"/>
+      <c r="I53" s="94" t="s">
+        <v>546</v>
+      </c>
+      <c r="J53" s="95" t="s">
         <v>164</v>
       </c>
-      <c r="K53" s="89"/>
-      <c r="L53" s="95" t="s">
-        <v>543</v>
-      </c>
-      <c r="M53" s="97"/>
-      <c r="N53" s="96"/>
-      <c r="O53" s="95"/>
-      <c r="P53" s="97"/>
-      <c r="Q53" s="95"/>
+      <c r="K53" s="90"/>
+      <c r="L53" s="96" t="s">
+        <v>547</v>
+      </c>
+      <c r="M53" s="98"/>
+      <c r="N53" s="97"/>
+      <c r="O53" s="96"/>
+      <c r="P53" s="98"/>
+      <c r="Q53" s="96"/>
       <c r="R53" s="58"/>
       <c r="U53" s="12"/>
       <c r="V53" s="59"/>
@@ -16350,20 +16378,20 @@
         <v>3</v>
       </c>
       <c r="E54" s="53" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="F54" s="13"/>
       <c r="G54" s="13"/>
       <c r="H54" s="13"/>
-      <c r="I54" s="87" t="s">
-        <v>545</v>
-      </c>
-      <c r="J54" s="88" t="s">
+      <c r="I54" s="88" t="s">
+        <v>549</v>
+      </c>
+      <c r="J54" s="89" t="s">
         <v>50</v>
       </c>
       <c r="K54" s="50"/>
       <c r="L54" s="56" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="M54" s="53" t="s">
         <v>108</v>
@@ -16386,36 +16414,36 @@
       <c r="AC54" s="63"/>
     </row>
     <row r="55" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="89" t="n">
+      <c r="B55" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C55" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D55" s="91" t="s">
+      <c r="C55" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D55" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E55" s="92" t="s">
-        <v>547</v>
-      </c>
-      <c r="F55" s="98"/>
-      <c r="G55" s="98"/>
-      <c r="H55" s="98"/>
-      <c r="I55" s="93" t="s">
-        <v>548</v>
-      </c>
-      <c r="J55" s="94" t="s">
+      <c r="E55" s="93" t="s">
+        <v>551</v>
+      </c>
+      <c r="F55" s="99"/>
+      <c r="G55" s="99"/>
+      <c r="H55" s="99"/>
+      <c r="I55" s="94" t="s">
+        <v>552</v>
+      </c>
+      <c r="J55" s="95" t="s">
         <v>164</v>
       </c>
-      <c r="K55" s="98"/>
-      <c r="L55" s="98" t="s">
-        <v>549</v>
-      </c>
-      <c r="M55" s="98"/>
-      <c r="N55" s="99"/>
-      <c r="O55" s="98"/>
-      <c r="P55" s="98"/>
-      <c r="Q55" s="98"/>
+      <c r="K55" s="99"/>
+      <c r="L55" s="99" t="s">
+        <v>553</v>
+      </c>
+      <c r="M55" s="99"/>
+      <c r="N55" s="100"/>
+      <c r="O55" s="99"/>
+      <c r="P55" s="99"/>
+      <c r="Q55" s="99"/>
     </row>
     <row r="56" customFormat="false" ht="32.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="50" t="n">
@@ -16428,16 +16456,16 @@
         <v>3</v>
       </c>
       <c r="E56" s="53" t="s">
-        <v>526</v>
-      </c>
-      <c r="I56" s="87" t="s">
-        <v>527</v>
-      </c>
-      <c r="J56" s="88" t="s">
-        <v>487</v>
+        <v>530</v>
+      </c>
+      <c r="I56" s="88" t="s">
+        <v>531</v>
+      </c>
+      <c r="J56" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L56" s="56" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="M56" s="53" t="s">
         <v>108</v>
@@ -16457,22 +16485,22 @@
         <v>3</v>
       </c>
       <c r="E57" s="53" t="s">
-        <v>550</v>
-      </c>
-      <c r="I57" s="87" t="s">
+        <v>554</v>
+      </c>
+      <c r="I57" s="88" t="s">
         <v>436</v>
       </c>
-      <c r="J57" s="88" t="s">
+      <c r="J57" s="89" t="s">
         <v>164</v>
       </c>
       <c r="L57" s="0" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="M57" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N57" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="32.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16486,16 +16514,16 @@
         <v>3</v>
       </c>
       <c r="E58" s="53" t="s">
-        <v>531</v>
-      </c>
-      <c r="I58" s="87" t="s">
-        <v>532</v>
-      </c>
-      <c r="J58" s="88" t="s">
-        <v>487</v>
+        <v>535</v>
+      </c>
+      <c r="I58" s="88" t="s">
+        <v>536</v>
+      </c>
+      <c r="J58" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L58" s="56" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="M58" s="53" t="s">
         <v>108</v>
@@ -16517,10 +16545,10 @@
       <c r="E59" s="53" t="s">
         <v>356</v>
       </c>
-      <c r="I59" s="87" t="s">
+      <c r="I59" s="88" t="s">
         <v>352</v>
       </c>
-      <c r="J59" s="88" t="s">
+      <c r="J59" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L59" s="0" t="s">
@@ -16542,22 +16570,22 @@
         <v>3</v>
       </c>
       <c r="E60" s="53" t="s">
-        <v>552</v>
-      </c>
-      <c r="I60" s="87" t="s">
-        <v>459</v>
-      </c>
-      <c r="J60" s="88" t="s">
+        <v>556</v>
+      </c>
+      <c r="I60" s="88" t="s">
+        <v>463</v>
+      </c>
+      <c r="J60" s="89" t="s">
         <v>164</v>
       </c>
       <c r="L60" s="0" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="M60" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N60" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="32.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16571,16 +16599,16 @@
         <v>3</v>
       </c>
       <c r="E61" s="53" t="s">
-        <v>534</v>
-      </c>
-      <c r="I61" s="87" t="s">
-        <v>535</v>
-      </c>
-      <c r="J61" s="88" t="s">
-        <v>487</v>
+        <v>538</v>
+      </c>
+      <c r="I61" s="88" t="s">
+        <v>539</v>
+      </c>
+      <c r="J61" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L61" s="56" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="M61" s="53" t="s">
         <v>108</v>
@@ -16600,16 +16628,16 @@
         <v>3</v>
       </c>
       <c r="E62" s="53" t="s">
-        <v>540</v>
-      </c>
-      <c r="I62" s="87" t="s">
-        <v>450</v>
-      </c>
-      <c r="J62" s="88" t="s">
-        <v>487</v>
+        <v>544</v>
+      </c>
+      <c r="I62" s="88" t="s">
+        <v>454</v>
+      </c>
+      <c r="J62" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L62" s="56" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="M62" s="86" t="s">
         <v>53</v>
@@ -16627,16 +16655,16 @@
         <v>3</v>
       </c>
       <c r="E63" s="53" t="s">
-        <v>554</v>
-      </c>
-      <c r="I63" s="87" t="s">
+        <v>558</v>
+      </c>
+      <c r="I63" s="88" t="s">
         <v>376</v>
       </c>
-      <c r="J63" s="88" t="s">
+      <c r="J63" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L63" s="0" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="M63" s="53" t="s">
         <v>108</v>
@@ -16646,36 +16674,36 @@
       </c>
     </row>
     <row r="64" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B64" s="89" t="n">
+      <c r="B64" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C64" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D64" s="91" t="s">
+      <c r="C64" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D64" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E64" s="92" t="s">
-        <v>541</v>
-      </c>
-      <c r="F64" s="98"/>
-      <c r="G64" s="98"/>
-      <c r="H64" s="98"/>
-      <c r="I64" s="93" t="s">
-        <v>542</v>
-      </c>
-      <c r="J64" s="94" t="s">
-        <v>487</v>
-      </c>
-      <c r="K64" s="98"/>
-      <c r="L64" s="95" t="s">
-        <v>543</v>
-      </c>
-      <c r="M64" s="98"/>
-      <c r="N64" s="99"/>
-      <c r="O64" s="98"/>
-      <c r="P64" s="98"/>
-      <c r="Q64" s="98"/>
+      <c r="E64" s="93" t="s">
+        <v>545</v>
+      </c>
+      <c r="F64" s="99"/>
+      <c r="G64" s="99"/>
+      <c r="H64" s="99"/>
+      <c r="I64" s="94" t="s">
+        <v>546</v>
+      </c>
+      <c r="J64" s="95" t="s">
+        <v>491</v>
+      </c>
+      <c r="K64" s="99"/>
+      <c r="L64" s="96" t="s">
+        <v>547</v>
+      </c>
+      <c r="M64" s="99"/>
+      <c r="N64" s="100"/>
+      <c r="O64" s="99"/>
+      <c r="P64" s="99"/>
+      <c r="Q64" s="99"/>
     </row>
     <row r="65" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B65" s="50" t="n">
@@ -16688,22 +16716,22 @@
         <v>3</v>
       </c>
       <c r="E65" s="53" t="s">
-        <v>556</v>
-      </c>
-      <c r="I65" s="87" t="s">
+        <v>560</v>
+      </c>
+      <c r="I65" s="88" t="s">
         <v>422</v>
       </c>
-      <c r="J65" s="88" t="s">
+      <c r="J65" s="89" t="s">
         <v>164</v>
       </c>
       <c r="L65" s="0" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="M65" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N65" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16717,52 +16745,52 @@
         <v>3</v>
       </c>
       <c r="E66" s="53" t="s">
-        <v>558</v>
-      </c>
-      <c r="I66" s="87" t="s">
-        <v>446</v>
-      </c>
-      <c r="J66" s="88" t="s">
+        <v>562</v>
+      </c>
+      <c r="I66" s="88" t="s">
+        <v>450</v>
+      </c>
+      <c r="J66" s="89" t="s">
         <v>164</v>
       </c>
       <c r="L66" s="0" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="M66" s="86" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B67" s="89" t="n">
+      <c r="B67" s="90" t="n">
         <v>1</v>
       </c>
-      <c r="C67" s="90" t="s">
-        <v>45</v>
-      </c>
-      <c r="D67" s="91" t="s">
+      <c r="C67" s="91" t="s">
+        <v>45</v>
+      </c>
+      <c r="D67" s="92" t="s">
         <v>62</v>
       </c>
-      <c r="E67" s="92" t="s">
-        <v>547</v>
-      </c>
-      <c r="F67" s="98"/>
-      <c r="G67" s="98"/>
-      <c r="H67" s="98"/>
-      <c r="I67" s="93" t="s">
-        <v>548</v>
-      </c>
-      <c r="J67" s="94" t="s">
-        <v>487</v>
-      </c>
-      <c r="K67" s="98"/>
-      <c r="L67" s="98" t="s">
-        <v>549</v>
-      </c>
-      <c r="M67" s="98"/>
-      <c r="N67" s="99"/>
-      <c r="O67" s="98"/>
-      <c r="P67" s="98"/>
-      <c r="Q67" s="98"/>
+      <c r="E67" s="93" t="s">
+        <v>551</v>
+      </c>
+      <c r="F67" s="99"/>
+      <c r="G67" s="99"/>
+      <c r="H67" s="99"/>
+      <c r="I67" s="94" t="s">
+        <v>552</v>
+      </c>
+      <c r="J67" s="95" t="s">
+        <v>491</v>
+      </c>
+      <c r="K67" s="99"/>
+      <c r="L67" s="99" t="s">
+        <v>553</v>
+      </c>
+      <c r="M67" s="99"/>
+      <c r="N67" s="100"/>
+      <c r="O67" s="99"/>
+      <c r="P67" s="99"/>
+      <c r="Q67" s="99"/>
     </row>
     <row r="68" customFormat="false" ht="32.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B68" s="50" t="n">
@@ -16775,22 +16803,22 @@
         <v>3</v>
       </c>
       <c r="E68" s="53" t="s">
-        <v>560</v>
-      </c>
-      <c r="I68" s="87" t="s">
+        <v>564</v>
+      </c>
+      <c r="I68" s="88" t="s">
         <v>378</v>
       </c>
-      <c r="J68" s="88" t="s">
+      <c r="J68" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L68" s="0" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="M68" s="0" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="N68" s="73" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16804,16 +16832,16 @@
         <v>3</v>
       </c>
       <c r="E69" s="53" t="s">
-        <v>550</v>
-      </c>
-      <c r="I69" s="87" t="s">
+        <v>554</v>
+      </c>
+      <c r="I69" s="88" t="s">
         <v>436</v>
       </c>
-      <c r="J69" s="88" t="s">
-        <v>487</v>
+      <c r="J69" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L69" s="0" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="M69" s="53" t="s">
         <v>329</v>
@@ -16831,16 +16859,16 @@
         <v>3</v>
       </c>
       <c r="E70" s="53" t="s">
-        <v>552</v>
-      </c>
-      <c r="I70" s="87" t="s">
-        <v>459</v>
-      </c>
-      <c r="J70" s="88" t="s">
-        <v>487</v>
+        <v>556</v>
+      </c>
+      <c r="I70" s="88" t="s">
+        <v>463</v>
+      </c>
+      <c r="J70" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L70" s="0" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="M70" s="53" t="s">
         <v>329</v>
@@ -16858,16 +16886,16 @@
         <v>3</v>
       </c>
       <c r="E71" s="53" t="s">
-        <v>564</v>
-      </c>
-      <c r="I71" s="87" t="s">
-        <v>565</v>
-      </c>
-      <c r="J71" s="88" t="s">
+        <v>568</v>
+      </c>
+      <c r="I71" s="88" t="s">
+        <v>569</v>
+      </c>
+      <c r="J71" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L71" s="0" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="M71" s="53" t="s">
         <v>108</v>
@@ -16887,22 +16915,22 @@
         <v>3</v>
       </c>
       <c r="E72" s="53" t="s">
-        <v>556</v>
-      </c>
-      <c r="I72" s="87" t="s">
+        <v>560</v>
+      </c>
+      <c r="I72" s="88" t="s">
         <v>422</v>
       </c>
-      <c r="J72" s="88" t="s">
-        <v>487</v>
+      <c r="J72" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L72" s="0" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="M72" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N72" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="32.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -16916,12 +16944,12 @@
         <v>3</v>
       </c>
       <c r="E73" s="53" t="s">
-        <v>567</v>
-      </c>
-      <c r="I73" s="87" t="s">
+        <v>571</v>
+      </c>
+      <c r="I73" s="88" t="s">
         <v>260</v>
       </c>
-      <c r="J73" s="88" t="s">
+      <c r="J73" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L73" s="0" t="s">
@@ -16945,16 +16973,16 @@
         <v>3</v>
       </c>
       <c r="E74" s="53" t="s">
-        <v>558</v>
-      </c>
-      <c r="I74" s="87" t="s">
-        <v>446</v>
-      </c>
-      <c r="J74" s="88" t="s">
-        <v>487</v>
+        <v>562</v>
+      </c>
+      <c r="I74" s="88" t="s">
+        <v>450</v>
+      </c>
+      <c r="J74" s="89" t="s">
+        <v>491</v>
       </c>
       <c r="L74" s="0" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="M74" s="86" t="s">
         <v>53</v>
@@ -16972,12 +17000,12 @@
         <v>3</v>
       </c>
       <c r="E75" s="53" t="s">
-        <v>569</v>
-      </c>
-      <c r="I75" s="87" t="s">
+        <v>573</v>
+      </c>
+      <c r="I75" s="88" t="s">
         <v>407</v>
       </c>
-      <c r="J75" s="88" t="s">
+      <c r="J75" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L75" s="0" t="s">
@@ -17001,22 +17029,22 @@
         <v>3</v>
       </c>
       <c r="E76" s="53" t="s">
-        <v>570</v>
-      </c>
-      <c r="I76" s="87" t="s">
+        <v>574</v>
+      </c>
+      <c r="I76" s="88" t="s">
         <v>384</v>
       </c>
-      <c r="J76" s="88" t="s">
+      <c r="J76" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L76" s="0" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="M76" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N76" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17030,22 +17058,22 @@
         <v>3</v>
       </c>
       <c r="E77" s="53" t="s">
-        <v>572</v>
-      </c>
-      <c r="I77" s="87" t="s">
+        <v>576</v>
+      </c>
+      <c r="I77" s="88" t="s">
         <v>411</v>
       </c>
-      <c r="J77" s="88" t="s">
+      <c r="J77" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L77" s="0" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="M77" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N77" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -17059,57 +17087,57 @@
         <v>3</v>
       </c>
       <c r="E78" s="53" t="s">
-        <v>574</v>
-      </c>
-      <c r="I78" s="87" t="s">
+        <v>578</v>
+      </c>
+      <c r="I78" s="88" t="s">
         <v>396</v>
       </c>
-      <c r="J78" s="88" t="s">
+      <c r="J78" s="89" t="s">
         <v>50</v>
       </c>
       <c r="L78" s="0" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="M78" s="53" t="s">
         <v>329</v>
       </c>
       <c r="N78" s="86" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="20.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B79" s="100" t="n">
+      <c r="B79" s="101" t="n">
         <v>1</v>
       </c>
-      <c r="C79" s="101" t="s">
-        <v>45</v>
-      </c>
-      <c r="D79" s="102" t="s">
+      <c r="C79" s="102" t="s">
+        <v>45</v>
+      </c>
+      <c r="D79" s="103" t="s">
         <v>62</v>
       </c>
-      <c r="E79" s="103" t="s">
-        <v>576</v>
-      </c>
-      <c r="F79" s="104"/>
-      <c r="G79" s="104"/>
-      <c r="H79" s="104"/>
-      <c r="I79" s="105" t="s">
-        <v>577</v>
-      </c>
-      <c r="J79" s="106" t="s">
+      <c r="E79" s="104" t="s">
+        <v>580</v>
+      </c>
+      <c r="F79" s="105"/>
+      <c r="G79" s="105"/>
+      <c r="H79" s="105"/>
+      <c r="I79" s="106" t="s">
+        <v>581</v>
+      </c>
+      <c r="J79" s="107" t="s">
         <v>50</v>
       </c>
-      <c r="K79" s="104"/>
-      <c r="L79" s="104" t="s">
-        <v>578</v>
-      </c>
-      <c r="M79" s="107" t="s">
+      <c r="K79" s="105"/>
+      <c r="L79" s="105" t="s">
+        <v>582</v>
+      </c>
+      <c r="M79" s="108" t="s">
         <v>108</v>
       </c>
-      <c r="N79" s="108"/>
-      <c r="O79" s="104"/>
-      <c r="P79" s="104"/>
-      <c r="Q79" s="104"/>
+      <c r="N79" s="109"/>
+      <c r="O79" s="105"/>
+      <c r="P79" s="105"/>
+      <c r="Q79" s="105"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -17228,39 +17256,39 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="12.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.0546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="115.2"/>
   </cols>
   <sheetData>
-    <row r="1" s="109" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="110" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="28" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="28" t="s">
-        <v>580</v>
-      </c>
-      <c r="B2" s="109"/>
+        <v>584</v>
+      </c>
+      <c r="B2" s="110"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="n">
         <v>14</v>
       </c>
-      <c r="B3" s="109"/>
+      <c r="B3" s="110"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28"/>
-      <c r="B4" s="109"/>
+      <c r="B4" s="110"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>580</v>
-      </c>
-      <c r="B5" s="109" t="s">
-        <v>581</v>
+        <v>584</v>
+      </c>
+      <c r="B5" s="110" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17268,7 +17296,7 @@
         <v>1</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17276,7 +17304,7 @@
         <v>2</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17284,7 +17312,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17292,7 +17320,7 @@
         <v>4</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17300,7 +17328,7 @@
         <v>5</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17308,7 +17336,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17316,7 +17344,7 @@
         <v>7</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17324,7 +17352,7 @@
         <v>8</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17332,7 +17360,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17340,7 +17368,7 @@
         <v>10</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17348,7 +17376,7 @@
         <v>11</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17356,7 +17384,7 @@
         <v>12</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="24.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17364,7 +17392,7 @@
         <v>13</v>
       </c>
       <c r="B18" s="86" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17372,7 +17400,7 @@
         <v>14</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
     </row>
   </sheetData>
@@ -17392,7 +17420,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -19749,7 +19777,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -21920,7 +21948,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -24388,7 +24416,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE30"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -25773,7 +25801,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -27949,7 +27977,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE30"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -29276,7 +29304,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE30"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>
@@ -30566,7 +30594,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:AE54"/>
-  <sheetFormatPr defaultColWidth="9.03125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="9.0390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="true" outlineLevel="0" max="1" min="1" style="0" width="11.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="10.01"/>

</xml_diff>